<commit_message>
Cleaned up the promotions excel file
</commit_message>
<xml_diff>
--- a/Assets/Promotions/promotion_com.spiraclestudios.autoskola.premium_186502.xlsx
+++ b/Assets/Promotions/promotion_com.spiraclestudios.autoskola.premium_186502.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Autoskola\Assets\Promotions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Autoskola\Assets\Promotions\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,94 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
-  <si>
-    <t>ZNDTPJJMG1HSH7HYWY71260</t>
-  </si>
-  <si>
-    <t>ZYDNP44BC6AMXC2MWKJSM7P</t>
-  </si>
-  <si>
-    <t>W9K8ZEEYZNC30WAQ7S76GXV</t>
-  </si>
-  <si>
-    <t>6EJXXKM6HZ0WE9WVN3LS1G8</t>
-  </si>
-  <si>
-    <t>AP2FXYQT9JRKNSHSS12W48J</t>
-  </si>
-  <si>
-    <t>9ED8LC4RBXSN85HFUQWD61P</t>
-  </si>
-  <si>
-    <t>TXA4KJYAWPAB32NXKH0P51X</t>
-  </si>
-  <si>
-    <t>3WL2HZ40XCMR22T5YCGSTXC</t>
-  </si>
-  <si>
-    <t>TNWQM9X1NBXN18LLR4CT7EQ</t>
-  </si>
-  <si>
-    <t>5Y0BE5UYJKETA7DPJNL1K3Y</t>
-  </si>
-  <si>
-    <t>8UXGZMW8JE0XVJ61NJ7Y34J</t>
-  </si>
-  <si>
-    <t>ZXBRQQ3PLJG21V9ZUSPTULZ</t>
-  </si>
-  <si>
-    <t>9FG94GL93S5EJS4YPVLKK2Q</t>
-  </si>
-  <si>
-    <t>CW40RZ7GEKJXHPA5MTGKFF0</t>
-  </si>
-  <si>
-    <t>JUGXG2PYEEE8TVRPYYR8DLV</t>
-  </si>
-  <si>
-    <t>LAK03GMCPW7H8NFVZNK3Q1N</t>
-  </si>
-  <si>
-    <t>BLPEF33SP2GDLAGGZ33PZMS</t>
-  </si>
-  <si>
-    <t>0U287M7R9D135EK20WM378B</t>
-  </si>
-  <si>
-    <t>TS8VUPXRVQTFCSLJ5AUHFBC</t>
-  </si>
-  <si>
-    <t>NEFT1RZAU56PJXPNBC37GKH</t>
-  </si>
-  <si>
-    <t>60UCZ1QFB8NDTNQSZDNB9NN</t>
-  </si>
-  <si>
-    <t>EA94GMS2GJL25SEX27SV56L</t>
-  </si>
-  <si>
-    <t>5PB70MCXTUY4U2U3VBKZU93</t>
-  </si>
-  <si>
-    <t>SHMMCX4R1AHM3NNRV64QEAN</t>
-  </si>
-  <si>
-    <t>Z27TFRN1W9PZSQNM7G60VP8</t>
-  </si>
-  <si>
-    <t>TJKTCR2H0D8UETT0EL71RUT</t>
-  </si>
-  <si>
-    <t>0TFRE29N246QHKSKKXC5RZT</t>
-  </si>
-  <si>
-    <t>G78X7X11DHEAC1TU26U1XR6</t>
-  </si>
-  <si>
-    <t>X5GQPDUCS014QMNFUCYG7T7</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>HWVXDZ4MXBQTDBEBZW3097R</t>
   </si>
@@ -141,101 +54,14 @@
     <t>4U9MXFFAF8HELHX9NG8799B</t>
   </si>
   <si>
-    <t>kamil.gore@azet.sk</t>
-  </si>
-  <si>
-    <t>lukas.nagy17@gmail.com</t>
-  </si>
-  <si>
-    <t>kwodo12@azet.sk </t>
-  </si>
-  <si>
-    <t>tiborbulak7141@gmail.com </t>
-  </si>
-  <si>
-    <t>ristemovicovaj@gmail.com </t>
-  </si>
-  <si>
-    <t>sristemovicova@gmail.com </t>
-  </si>
-  <si>
-    <t>5c1debnarova@gmail.com</t>
-  </si>
-  <si>
-    <t>misohari@azet.sk</t>
-  </si>
-  <si>
-    <t>darius.petruska@azet.sk</t>
-  </si>
-  <si>
-    <t>lukas.krupcik@gmail.com</t>
-  </si>
-  <si>
-    <t>Erik513@azet.sk</t>
-  </si>
-  <si>
-    <t>p.samel@centrum.sk</t>
-  </si>
-  <si>
-    <t>2pac-e@azet.sk</t>
-  </si>
-  <si>
-    <t>kaja21101@azet.sk</t>
-  </si>
-  <si>
-    <t>milos02713@azet.sk</t>
-  </si>
-  <si>
-    <t>zuzana.novakiova@gmail.com</t>
-  </si>
-  <si>
-    <t>vanesakockova05@gmail.com</t>
-  </si>
-  <si>
-    <t>stevo.ziga12@zoznam.sk</t>
-  </si>
-  <si>
-    <t>natali1584@azet.sk</t>
-  </si>
-  <si>
-    <t>angelika.aja.123@gmail.com</t>
-  </si>
-  <si>
-    <t>aoetaki@gmail.com</t>
-  </si>
-  <si>
-    <t>vikinanovotna@gmail.com</t>
-  </si>
-  <si>
-    <t>majk992304@gmail.com</t>
-  </si>
-  <si>
-    <t>kuncik221@azet.sk</t>
-  </si>
-  <si>
-    <t>miselka.mi@gmail.com</t>
-  </si>
-  <si>
-    <t>anetka.boberova@gmail.com</t>
-  </si>
-  <si>
-    <t>lydia232@centrum.sk</t>
-  </si>
-  <si>
-    <t>lucia316@centrum.sk</t>
-  </si>
-  <si>
-    <t>benjiko99@gmail.com</t>
-  </si>
-  <si>
-    <t>martiny used it</t>
+    <t>Unused promo codes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +202,15 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -721,10 +556,13 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="7" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -753,7 +591,6 @@
     <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -761,6 +598,7 @@
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -1047,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
@@ -1055,329 +893,131 @@
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
-      </c>
+    <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>41</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>42</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>43</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>44</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>45</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B6" s="1"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>46</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B7" s="1"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>47</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B8" s="1"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B9" s="1"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>49</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B10" s="1"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>50</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B11" s="1"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>51</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B12" s="1"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>52</v>
-      </c>
+      <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>53</v>
-      </c>
+      <c r="B14" s="1"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>54</v>
-      </c>
+      <c r="B15" s="1"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C29" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
+      <c r="B16" s="1"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1"/>
-    <hyperlink ref="B10" r:id="rId2"/>
-    <hyperlink ref="B9" r:id="rId3"/>
-    <hyperlink ref="B8" r:id="rId4"/>
-    <hyperlink ref="B6" r:id="rId5"/>
-    <hyperlink ref="B7" r:id="rId6"/>
-    <hyperlink ref="B5" r:id="rId7"/>
-    <hyperlink ref="B4" r:id="rId8"/>
-    <hyperlink ref="B3" r:id="rId9"/>
-    <hyperlink ref="B2" r:id="rId10"/>
-    <hyperlink ref="B1" r:id="rId11"/>
-    <hyperlink ref="B12" r:id="rId12"/>
-    <hyperlink ref="B13" r:id="rId13"/>
-    <hyperlink ref="B14" r:id="rId14"/>
-    <hyperlink ref="B15" r:id="rId15"/>
-    <hyperlink ref="B16" r:id="rId16"/>
-    <hyperlink ref="B17" r:id="rId17"/>
-    <hyperlink ref="B18" r:id="rId18"/>
-    <hyperlink ref="B19" r:id="rId19"/>
-    <hyperlink ref="B20" r:id="rId20"/>
-    <hyperlink ref="B21" r:id="rId21"/>
-    <hyperlink ref="B22" r:id="rId22"/>
-    <hyperlink ref="B23" r:id="rId23"/>
-    <hyperlink ref="B24" r:id="rId24"/>
-    <hyperlink ref="B25" r:id="rId25"/>
-    <hyperlink ref="B26" r:id="rId26"/>
-    <hyperlink ref="B27" r:id="rId27"/>
-    <hyperlink ref="B28" r:id="rId28"/>
-    <hyperlink ref="B29" r:id="rId29"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId30"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>